<commit_message>
Fix recursive benchmark anchor calibration
</commit_message>
<xml_diff>
--- a/Thesis Forecasting/outputs/random_forest_forecast/Day_Ahead_24H_RANDOM_FOREST.xlsx
+++ b/Thesis Forecasting/outputs/random_forest_forecast/Day_Ahead_24H_RANDOM_FOREST.xlsx
@@ -640,13 +640,13 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>47.41614715248679</v>
+        <v>47.29365542531561</v>
       </c>
       <c r="P2" t="n">
-        <v>28.321941349568</v>
+        <v>28.24877632623549</v>
       </c>
       <c r="Q2" t="n">
-        <v>48.08441149794521</v>
+        <v>47.96019342102194</v>
       </c>
       <c r="R2" t="n">
         <v>21.81494466535429</v>
@@ -667,13 +667,13 @@
         <v>43.13001582680973</v>
       </c>
       <c r="X2" t="n">
-        <v>158.3225</v>
+        <v>158.002625172573</v>
       </c>
       <c r="Y2" t="n">
         <v>43.37393297984622</v>
       </c>
       <c r="Z2" t="n">
-        <v>575.3397518733947</v>
+        <v>575.0198770459677</v>
       </c>
     </row>
     <row r="3">
@@ -722,10 +722,10 @@
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>44.87902252362228</v>
+        <v>44.87093680695329</v>
       </c>
       <c r="P3" t="n">
-        <v>26.66202747637768</v>
+        <v>26.657155053483</v>
       </c>
       <c r="Q3" t="n">
         <v>50</v>
@@ -749,13 +749,13 @@
         <v>42.59741851679561</v>
       </c>
       <c r="X3" t="n">
-        <v>156.04105</v>
+        <v>156.0280918604363</v>
       </c>
       <c r="Y3" t="n">
         <v>42.15495845990617</v>
       </c>
       <c r="Z3" t="n">
-        <v>570.4285893666587</v>
+        <v>570.4156312270951</v>
       </c>
     </row>
     <row r="4">
@@ -804,10 +804,10 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>46.91721250332506</v>
+        <v>46.54958392792987</v>
       </c>
       <c r="P4" t="n">
-        <v>26.11041249667492</v>
+        <v>25.90561831054565</v>
       </c>
       <c r="Q4" t="n">
         <v>50</v>
@@ -831,13 +831,13 @@
         <v>42.62680687164975</v>
       </c>
       <c r="X4" t="n">
-        <v>157.527625</v>
+        <v>156.9552022384755</v>
       </c>
       <c r="Y4" t="n">
         <v>41.6885368018397</v>
       </c>
       <c r="Z4" t="n">
-        <v>571.8290479380728</v>
+        <v>571.2566251765484</v>
       </c>
     </row>
     <row r="5">
@@ -886,10 +886,10 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>47.61289949852959</v>
+        <v>47.20093886531757</v>
       </c>
       <c r="P5" t="n">
-        <v>25.75461300147043</v>
+        <v>25.52900147605483</v>
       </c>
       <c r="Q5" t="n">
         <v>50</v>
@@ -913,13 +913,13 @@
         <v>43.29704688831825</v>
       </c>
       <c r="X5" t="n">
-        <v>157.8675125</v>
+        <v>157.2299403413724</v>
       </c>
       <c r="Y5" t="n">
         <v>41.09865364806093</v>
       </c>
       <c r="Z5" t="n">
-        <v>571.1976489716906</v>
+        <v>570.560076813063</v>
       </c>
     </row>
     <row r="6">
@@ -968,10 +968,10 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>48.31246961784986</v>
+        <v>47.90298452929319</v>
       </c>
       <c r="P6" t="n">
-        <v>25.01253663215013</v>
+        <v>24.79393097127604</v>
       </c>
       <c r="Q6" t="n">
         <v>50</v>
@@ -995,13 +995,13 @@
         <v>43.83899226414883</v>
       </c>
       <c r="X6" t="n">
-        <v>157.82500625</v>
+        <v>157.1969155005692</v>
       </c>
       <c r="Y6" t="n">
         <v>40.23018138278884</v>
       </c>
       <c r="Z6" t="n">
-        <v>570.1434364607849</v>
+        <v>569.5153457113541</v>
       </c>
     </row>
     <row r="7">
@@ -1050,19 +1050,19 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>48.70607997557301</v>
+        <v>48.32472719083246</v>
       </c>
       <c r="P7" t="n">
-        <v>24.29267314942699</v>
+        <v>24.0934956963459</v>
       </c>
       <c r="Q7" t="n">
         <v>50</v>
       </c>
       <c r="R7" t="n">
-        <v>19.85929471779943</v>
+        <v>19.86059100765223</v>
       </c>
       <c r="S7" t="n">
-        <v>19.51300652625513</v>
+        <v>19.51428021259279</v>
       </c>
       <c r="T7" t="n">
         <v>60.27303760684958</v>
@@ -1077,13 +1077,13 @@
         <v>43.52469005319531</v>
       </c>
       <c r="X7" t="n">
-        <v>157.498753125</v>
+        <v>156.9182228871784</v>
       </c>
       <c r="Y7" t="n">
-        <v>39.37230124405455</v>
+        <v>39.37487122024503</v>
       </c>
       <c r="Z7" t="n">
-        <v>568.159538309407</v>
+        <v>567.5815780477758</v>
       </c>
     </row>
     <row r="8">
@@ -1132,19 +1132,19 @@
         <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>49.37897687737681</v>
+        <v>48.95109085790975</v>
       </c>
       <c r="P8" t="n">
-        <v>23.81494968512318</v>
+        <v>23.5983242514585</v>
       </c>
       <c r="Q8" t="n">
         <v>50</v>
       </c>
       <c r="R8" t="n">
-        <v>20.50823934536045</v>
+        <v>20.50953583313301</v>
       </c>
       <c r="S8" t="n">
-        <v>20.14442853303628</v>
+        <v>20.14570202145419</v>
       </c>
       <c r="T8" t="n">
         <v>59.45274353405233</v>
@@ -1159,13 +1159,13 @@
         <v>43.84857740728881</v>
       </c>
       <c r="X8" t="n">
-        <v>157.6939265625</v>
+        <v>157.0494151093683</v>
       </c>
       <c r="Y8" t="n">
-        <v>40.65266787839673</v>
+        <v>40.65523785458721</v>
       </c>
       <c r="Z8" t="n">
-        <v>568.4649209920755</v>
+        <v>567.8229795151341</v>
       </c>
     </row>
     <row r="9">
@@ -1217,16 +1217,16 @@
         <v>50</v>
       </c>
       <c r="P9" t="n">
-        <v>23.85657506408953</v>
+        <v>23.51624119024137</v>
       </c>
       <c r="Q9" t="n">
-        <v>49.67493821716049</v>
+        <v>49.34650449445244</v>
       </c>
       <c r="R9" t="n">
-        <v>20.75344629631367</v>
+        <v>20.75474199941669</v>
       </c>
       <c r="S9" t="n">
-        <v>20.41019893030716</v>
+        <v>20.41147320339461</v>
       </c>
       <c r="T9" t="n">
         <v>59.47831404564473</v>
@@ -1241,13 +1241,13 @@
         <v>44.23957245527882</v>
       </c>
       <c r="X9" t="n">
-        <v>158.03151328125</v>
+        <v>157.3627456846938</v>
       </c>
       <c r="Y9" t="n">
-        <v>41.16364522662083</v>
+        <v>41.1662152028113</v>
       </c>
       <c r="Z9" t="n">
-        <v>569.1254937311235</v>
+        <v>568.4592961107577</v>
       </c>
     </row>
     <row r="10">
@@ -1296,19 +1296,19 @@
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>48.12695120493856</v>
+        <v>47.93231638472174</v>
       </c>
       <c r="P10" t="n">
-        <v>25.18005543568642</v>
+        <v>24.77397277631962</v>
       </c>
       <c r="Q10" t="n">
         <v>50</v>
       </c>
       <c r="R10" t="n">
-        <v>20.78374734083666</v>
+        <v>20.79058197397271</v>
       </c>
       <c r="S10" t="n">
-        <v>20.31931049276</v>
+        <v>20.32599239812182</v>
       </c>
       <c r="T10" t="n">
         <v>59.1491458255686</v>
@@ -1323,13 +1323,13 @@
         <v>44.26375516129129</v>
       </c>
       <c r="X10" t="n">
-        <v>157.807006640625</v>
+        <v>157.2062891610414</v>
       </c>
       <c r="Y10" t="n">
-        <v>41.10305783359666</v>
+        <v>41.11657437209453</v>
       </c>
       <c r="Z10" t="n">
-        <v>567.9842884909364</v>
+        <v>567.3970875498507</v>
       </c>
     </row>
     <row r="11">
@@ -1378,19 +1378,19 @@
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>48.03411818653069</v>
+        <v>47.8389727151766</v>
       </c>
       <c r="P11" t="n">
-        <v>25.1314851337818</v>
+        <v>24.72572779876435</v>
       </c>
       <c r="Q11" t="n">
         <v>50</v>
       </c>
       <c r="R11" t="n">
-        <v>20.49036589849551</v>
+        <v>20.50278208098408</v>
       </c>
       <c r="S11" t="n">
-        <v>20.03257747308037</v>
+        <v>20.04471625766109</v>
       </c>
       <c r="T11" t="n">
         <v>59.34350979545975</v>
@@ -1405,13 +1405,13 @@
         <v>44.15756596091144</v>
       </c>
       <c r="X11" t="n">
-        <v>157.6656033203125</v>
+        <v>157.0647005139409</v>
       </c>
       <c r="Y11" t="n">
-        <v>40.52294337157588</v>
+        <v>40.54749833864518</v>
       </c>
       <c r="Z11" t="n">
-        <v>566.8429738126561</v>
+        <v>566.2666259733537</v>
       </c>
     </row>
     <row r="12">
@@ -1460,19 +1460,19 @@
         <v>0</v>
       </c>
       <c r="O12" t="n">
-        <v>48.07521476631519</v>
+        <v>47.87087749365148</v>
       </c>
       <c r="P12" t="n">
-        <v>25.15298689384103</v>
+        <v>24.74221788672562</v>
       </c>
       <c r="Q12" t="n">
         <v>50</v>
       </c>
       <c r="R12" t="n">
-        <v>20.44576038852941</v>
+        <v>20.45750320695243</v>
       </c>
       <c r="S12" t="n">
-        <v>19.86766234619489</v>
+        <v>19.87907313977692</v>
       </c>
       <c r="T12" t="n">
         <v>59.21687322848535</v>
@@ -1487,13 +1487,13 @@
         <v>44.1224521570871</v>
       </c>
       <c r="X12" t="n">
-        <v>157.7282016601562</v>
+        <v>157.1130953803771</v>
       </c>
       <c r="Y12" t="n">
-        <v>40.3134227347243</v>
+        <v>40.33657634672935</v>
       </c>
       <c r="Z12" t="n">
-        <v>566.1416888402816</v>
+        <v>565.5497361725074</v>
       </c>
     </row>
     <row r="13">
@@ -1542,19 +1542,19 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>48.2374712351884</v>
+        <v>48.02355688214644</v>
       </c>
       <c r="P13" t="n">
-        <v>25.23787959488973</v>
+        <v>24.82113072256105</v>
       </c>
       <c r="Q13" t="n">
         <v>50</v>
       </c>
       <c r="R13" t="n">
-        <v>20.88951744344029</v>
+        <v>20.89706166498817</v>
       </c>
       <c r="S13" t="n">
-        <v>20.21515973678024</v>
+        <v>20.22246041493583</v>
       </c>
       <c r="T13" t="n">
         <v>59.36619013368323</v>
@@ -1569,13 +1569,13 @@
         <v>44.08529262796475</v>
       </c>
       <c r="X13" t="n">
-        <v>157.9753508300781</v>
+        <v>157.3446876047075</v>
       </c>
       <c r="Y13" t="n">
-        <v>41.10467718022053</v>
+        <v>41.119522079924</v>
       </c>
       <c r="Z13" t="n">
-        <v>566.8818165612695</v>
+        <v>566.2659982356023</v>
       </c>
     </row>
     <row r="14">
@@ -1624,19 +1624,19 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>46.53126115796824</v>
+        <v>46.58531990520488</v>
       </c>
       <c r="P14" t="n">
-        <v>24.34518925707083</v>
+        <v>24.07777328857725</v>
       </c>
       <c r="Q14" t="n">
         <v>50</v>
       </c>
       <c r="R14" t="n">
-        <v>21.34304891619041</v>
+        <v>21.360025347447</v>
       </c>
       <c r="S14" t="n">
-        <v>20.63625208439357</v>
+        <v>20.6526663238155</v>
       </c>
       <c r="T14" t="n">
         <v>58.9421976541837</v>
@@ -1651,13 +1651,13 @@
         <v>44.0154453249852</v>
       </c>
       <c r="X14" t="n">
-        <v>155.3764504150391</v>
+        <v>155.1630931937821</v>
       </c>
       <c r="Y14" t="n">
-        <v>41.97930100058398</v>
+        <v>42.0126916712625</v>
       </c>
       <c r="Z14" t="n">
-        <v>564.4191267021399</v>
+        <v>564.2391601515615</v>
       </c>
     </row>
     <row r="15">
@@ -1706,19 +1706,19 @@
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>47.34541833217028</v>
+        <v>47.0799012828821</v>
       </c>
       <c r="P15" t="n">
-        <v>24.77115687534924</v>
+        <v>24.33339927351621</v>
       </c>
       <c r="Q15" t="n">
         <v>50</v>
       </c>
       <c r="R15" t="n">
-        <v>21.17368456676961</v>
+        <v>21.19059067998293</v>
       </c>
       <c r="S15" t="n">
-        <v>20.41659958805299</v>
+        <v>20.43290120730958</v>
       </c>
       <c r="T15" t="n">
         <v>58.48216465976965</v>
@@ -1733,13 +1733,13 @@
         <v>43.97448452515925</v>
       </c>
       <c r="X15" t="n">
-        <v>156.6165752075195</v>
+        <v>155.9133005563983</v>
       </c>
       <c r="Y15" t="n">
-        <v>41.5902841548226</v>
+        <v>41.6234918872925</v>
       </c>
       <c r="Z15" t="n">
-        <v>564.5506943611898</v>
+        <v>563.8806274425385</v>
       </c>
     </row>
     <row r="16">
@@ -1788,19 +1788,19 @@
         <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>47.81296170168567</v>
+        <v>47.53863050063595</v>
       </c>
       <c r="P16" t="n">
-        <v>25.01577590207406</v>
+        <v>24.57049495362314</v>
       </c>
       <c r="Q16" t="n">
         <v>50</v>
       </c>
       <c r="R16" t="n">
-        <v>20.9663678938729</v>
+        <v>20.9838858413281</v>
       </c>
       <c r="S16" t="n">
-        <v>20.29624850327781</v>
+        <v>20.31320654849659</v>
       </c>
       <c r="T16" t="n">
         <v>58.97369094234622</v>
@@ -1815,13 +1815,13 @@
         <v>43.97252295949446</v>
       </c>
       <c r="X16" t="n">
-        <v>157.3287376037597</v>
+        <v>156.6091254542591</v>
       </c>
       <c r="Y16" t="n">
-        <v>41.26261639715071</v>
+        <v>41.29709238982468</v>
       </c>
       <c r="Z16" t="n">
-        <v>565.1847360810542</v>
+        <v>564.4995999242274</v>
       </c>
     </row>
     <row r="17">
@@ -1870,19 +1870,19 @@
         <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>47.03471229194007</v>
+        <v>46.78276922888862</v>
       </c>
       <c r="P17" t="n">
-        <v>26.31630650993981</v>
+        <v>25.88037739530789</v>
       </c>
       <c r="Q17" t="n">
         <v>50</v>
       </c>
       <c r="R17" t="n">
-        <v>20.71791592185287</v>
+        <v>20.73136398458464</v>
       </c>
       <c r="S17" t="n">
-        <v>20.15105334845808</v>
+        <v>20.16413345895584</v>
       </c>
       <c r="T17" t="n">
         <v>58.80803447134171</v>
@@ -1897,13 +1897,13 @@
         <v>43.97270651406613</v>
       </c>
       <c r="X17" t="n">
-        <v>157.8510188018799</v>
+        <v>157.1631466241965</v>
       </c>
       <c r="Y17" t="n">
-        <v>40.86896927031095</v>
+        <v>40.89549744354048</v>
       </c>
       <c r="Z17" t="n">
-        <v>564.9379860787824</v>
+        <v>564.2766420743285</v>
       </c>
     </row>
     <row r="18">
@@ -1952,19 +1952,19 @@
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>43.61213266161683</v>
+        <v>43.41756261036799</v>
       </c>
       <c r="P18" t="n">
-        <v>29.8479267393231</v>
+        <v>29.44646161489149</v>
       </c>
       <c r="Q18" t="n">
         <v>50</v>
       </c>
       <c r="R18" t="n">
-        <v>20.5882423806537</v>
+        <v>20.60023122466999</v>
       </c>
       <c r="S18" t="n">
-        <v>20.02472021340295</v>
+        <v>20.03638090996313</v>
       </c>
       <c r="T18" t="n">
         <v>59.06566162214764</v>
@@ -1979,13 +1979,13 @@
         <v>43.97029627075541</v>
       </c>
       <c r="X18" t="n">
-        <v>157.9600594009399</v>
+        <v>157.3640242252595</v>
       </c>
       <c r="Y18" t="n">
-        <v>40.61296259405664</v>
+        <v>40.63661213463313</v>
       </c>
       <c r="Z18" t="n">
-        <v>564.839338929614</v>
+        <v>564.26695329451</v>
       </c>
     </row>
     <row r="19">
@@ -2034,19 +2034,19 @@
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>42.32695983160359</v>
+        <v>42.1751873138739</v>
       </c>
       <c r="P19" t="n">
-        <v>31.00096986886637</v>
+        <v>30.65624955418724</v>
       </c>
       <c r="Q19" t="n">
         <v>50</v>
       </c>
       <c r="R19" t="n">
-        <v>20.59895868186451</v>
+        <v>20.60858546403213</v>
       </c>
       <c r="S19" t="n">
-        <v>19.98578302416482</v>
+        <v>19.99512324289114</v>
       </c>
       <c r="T19" t="n">
         <v>59.47288203796191</v>
@@ -2061,13 +2061,13 @@
         <v>43.97412765661268</v>
       </c>
       <c r="X19" t="n">
-        <v>157.82792970047</v>
+        <v>157.3314368680611</v>
       </c>
       <c r="Y19" t="n">
-        <v>40.58474170602932</v>
+        <v>40.60370870692327</v>
       </c>
       <c r="Z19" t="n">
-        <v>564.8831421633188</v>
+        <v>564.4056163318039</v>
       </c>
     </row>
     <row r="20">
@@ -2116,19 +2116,19 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>42.84830177117978</v>
+        <v>42.69482018911886</v>
       </c>
       <c r="P20" t="n">
-        <v>30.42941307905521</v>
+        <v>30.12399885741173</v>
       </c>
       <c r="Q20" t="n">
         <v>50</v>
       </c>
       <c r="R20" t="n">
-        <v>20.87683526159622</v>
+        <v>20.88415871791736</v>
       </c>
       <c r="S20" t="n">
-        <v>20.23555979578988</v>
+        <v>20.24265829690086</v>
       </c>
       <c r="T20" t="n">
         <v>59.12592368747497</v>
@@ -2143,13 +2143,13 @@
         <v>43.96744325744439</v>
       </c>
       <c r="X20" t="n">
-        <v>157.777714850235</v>
+        <v>157.3188190465306</v>
       </c>
       <c r="Y20" t="n">
-        <v>41.1123950573861</v>
+        <v>41.12681701481822</v>
       </c>
       <c r="Z20" t="n">
-        <v>564.8000399353159</v>
+        <v>564.3555660890438</v>
       </c>
     </row>
     <row r="21">
@@ -2198,19 +2198,19 @@
         <v>0</v>
       </c>
       <c r="O21" t="n">
-        <v>43.31719562114957</v>
+        <v>43.14203348254161</v>
       </c>
       <c r="P21" t="n">
-        <v>29.97711180396793</v>
+        <v>29.69051370819313</v>
       </c>
       <c r="Q21" t="n">
         <v>50</v>
       </c>
       <c r="R21" t="n">
-        <v>21.16928592322156</v>
+        <v>21.16820155108741</v>
       </c>
       <c r="S21" t="n">
-        <v>20.50708409128169</v>
+        <v>20.50603363966882</v>
       </c>
       <c r="T21" t="n">
         <v>59.16479512178694</v>
@@ -2225,13 +2225,13 @@
         <v>43.97130251936676</v>
       </c>
       <c r="X21" t="n">
-        <v>157.7943074251175</v>
+        <v>157.3325471907347</v>
       </c>
       <c r="Y21" t="n">
-        <v>41.67637001450325</v>
+        <v>41.67423519075624</v>
       </c>
       <c r="Z21" t="n">
-        <v>565.214990717454</v>
+        <v>564.7510956593242</v>
       </c>
     </row>
     <row r="22">
@@ -2280,19 +2280,19 @@
         <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>43.6784184084262</v>
+        <v>43.48618230937074</v>
       </c>
       <c r="P22" t="n">
-        <v>29.57253530413255</v>
+        <v>29.30297577927797</v>
       </c>
       <c r="Q22" t="n">
         <v>50</v>
       </c>
       <c r="R22" t="n">
-        <v>21.01129929293297</v>
+        <v>21.01057010968128</v>
       </c>
       <c r="S22" t="n">
-        <v>20.33804391936124</v>
+        <v>20.33733810099221</v>
       </c>
       <c r="T22" t="n">
         <v>59.62444504751775</v>
@@ -2307,13 +2307,13 @@
         <v>44.01634052966378</v>
       </c>
       <c r="X22" t="n">
-        <v>157.7509537125588</v>
+        <v>157.2891580886487</v>
       </c>
       <c r="Y22" t="n">
-        <v>41.34934321229422</v>
+        <v>41.34790821067349</v>
       </c>
       <c r="Z22" t="n">
-        <v>565.1465958178549</v>
+        <v>564.6833651923241</v>
       </c>
     </row>
     <row r="23">
@@ -2362,19 +2362,19 @@
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>43.89111634717568</v>
+        <v>43.69770825698051</v>
       </c>
       <c r="P23" t="n">
-        <v>29.18231050910368</v>
+        <v>28.93624794885192</v>
       </c>
       <c r="Q23" t="n">
         <v>50</v>
       </c>
       <c r="R23" t="n">
-        <v>20.73297486223188</v>
+        <v>20.73341334098356</v>
       </c>
       <c r="S23" t="n">
-        <v>20.1892813390492</v>
+        <v>20.18970831930348</v>
       </c>
       <c r="T23" t="n">
         <v>58.85169522734232</v>
@@ -2389,13 +2389,13 @@
         <v>44.01131976456341</v>
       </c>
       <c r="X23" t="n">
-        <v>157.5734268562794</v>
+        <v>157.1339562058324</v>
       </c>
       <c r="Y23" t="n">
-        <v>40.92225620128109</v>
+        <v>40.92312166028704</v>
       </c>
       <c r="Z23" t="n">
-        <v>563.5615090444275</v>
+        <v>563.1229038529865</v>
       </c>
     </row>
     <row r="24">
@@ -2444,19 +2444,19 @@
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>44.22439834206929</v>
+        <v>44.00046198659694</v>
       </c>
       <c r="P24" t="n">
-        <v>28.96436508607037</v>
+        <v>28.71837511468768</v>
       </c>
       <c r="Q24" t="n">
         <v>50</v>
       </c>
       <c r="R24" t="n">
-        <v>20.52538666662094</v>
+        <v>20.52194025200813</v>
       </c>
       <c r="S24" t="n">
-        <v>20.03521457349928</v>
+        <v>20.03185046360949</v>
       </c>
       <c r="T24" t="n">
         <v>59.53183172936171</v>
@@ -2471,13 +2471,13 @@
         <v>43.97728454846853</v>
       </c>
       <c r="X24" t="n">
-        <v>157.6887634281397</v>
+        <v>157.2188371012846</v>
       </c>
       <c r="Y24" t="n">
-        <v>40.56060124012022</v>
+        <v>40.55379071561762</v>
       </c>
       <c r="Z24" t="n">
-        <v>563.7600390868191</v>
+        <v>563.2833022354615</v>
       </c>
     </row>
     <row r="25">
@@ -2526,19 +2526,19 @@
         <v>0</v>
       </c>
       <c r="O25" t="n">
-        <v>44.41877415118671</v>
+        <v>44.20174007253119</v>
       </c>
       <c r="P25" t="n">
-        <v>28.69225756288314</v>
+        <v>28.4679969648526</v>
       </c>
       <c r="Q25" t="n">
         <v>50</v>
       </c>
       <c r="R25" t="n">
-        <v>20.41674724841148</v>
+        <v>20.40971500599191</v>
       </c>
       <c r="S25" t="n">
-        <v>19.96388915899053</v>
+        <v>19.95701289674877</v>
       </c>
       <c r="T25" t="n">
         <v>59.83262576504894</v>
@@ -2553,13 +2553,13 @@
         <v>43.93544988599814</v>
       </c>
       <c r="X25" t="n">
-        <v>157.6110317140698</v>
+        <v>157.1697370373838</v>
       </c>
       <c r="Y25" t="n">
-        <v>40.38063640740201</v>
+        <v>40.36672790274068</v>
       </c>
       <c r="Z25" t="n">
-        <v>563.4606913487156</v>
+        <v>563.0054881673682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>